<commit_message>
Industec: admin@industec.com.au added to the To
Andrew's address for them, 3 Aug 2026.

Added ALONGSIDE m.clayton@industec.com.au rather than replacing it.
That one came out of the routing workbook, and dropping a contact
nobody asked me to drop is not mine to decide quietly - asked him
which he wants.

Industec Filtration now reads:
    TO  m.clayton@industec.com.au, admin@industec.com.au
    CC  Pickels, Moore, Vandenbroek, Maher, Mitchell

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cvkBVSy5jN5HGmHFYEnYK
</commit_message>
<xml_diff>
--- a/01_Reporting_Suite/Coates_Report_Recipients.xlsx
+++ b/01_Reporting_Suite/Coates_Report_Recipients.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3929,6 +3929,43 @@
       <c r="G98" t="inlineStr">
         <is>
           <t>Coates - standing Cc on every company report (Andrew, 3 Aug 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Industec Filtration</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Industec admin</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>admin@industec.com.au</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>COMPANY,DEMOB</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Site contact - Andrew, 3 Aug 2026</t>
         </is>
       </c>
     </row>

</xml_diff>